<commit_message>
changes to add missing data column and allow data to save even if missing
</commit_message>
<xml_diff>
--- a/climate_trace_tools/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
+++ b/climate_trace_tools/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
@@ -3772,8 +3772,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D3" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.ii Combined Heat and Power Generation")</f>
-        <v>1.A.1.a.ii Combined Heat and Power Generation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.ii  Combined Heat and Power Generation")</f>
+        <v>1.A.1.a.ii  Combined Heat and Power Generation</v>
       </c>
       <c r="E3" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3799,8 +3799,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D4" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii Heat Plants")</f>
-        <v>1.A.1.a.iii Heat Plants</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii  Heat Plants")</f>
+        <v>1.A.1.a.iii  Heat Plants</v>
       </c>
       <c r="E4" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4042,8 +4042,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D13" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.5 Other (Not specified elsewhere)")</f>
-        <v>1.A.5 Other (Not specified elsewhere)</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.5  Other (Not specified elsewhere)")</f>
+        <v>1.A.5  Other (Not specified elsewhere)</v>
       </c>
       <c r="E13" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4474,8 +4474,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D29" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi Other")</f>
-        <v>1.B.2.b.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi  Other")</f>
+        <v>1.B.2.b.vi  Other</v>
       </c>
       <c r="E29" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4501,8 +4501,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D30" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi Other")</f>
-        <v>1.B.2.a.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi  Other")</f>
+        <v>1.B.2.a.vi  Other</v>
       </c>
       <c r="E30" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4528,8 +4528,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D31" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.d Other")</f>
-        <v>1.B.2.d Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.d  Other")</f>
+        <v>1.B.2.d  Other</v>
       </c>
       <c r="E31" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4771,8 +4771,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D40" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.a Methanol")</f>
-        <v>2.B.8.a Methanol</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.a  Methanol")</f>
+        <v>2.B.8.a  Methanol</v>
       </c>
       <c r="E40" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4798,8 +4798,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D41" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.7 Soda Ash Production")</f>
-        <v>2.B.7 Soda Ash Production</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.7  Soda Ash Production")</f>
+        <v>2.B.7  Soda Ash Production</v>
       </c>
       <c r="E41" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4825,8 +4825,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D42" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c Chemicals")</f>
-        <v>1.A.2.c Chemicals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
       </c>
       <c r="E42" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -5068,8 +5068,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D51" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c Chemicals")</f>
-        <v>1.A.2.c Chemicals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
       </c>
       <c r="E51" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -5257,8 +5257,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D58" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.a Methanol")</f>
-        <v>2.B.8.a Methanol</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.a  Methanol")</f>
+        <v>2.B.8.a  Methanol</v>
       </c>
       <c r="E58" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -5284,8 +5284,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D59" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.7 Soda Ash Production")</f>
-        <v>2.B.7 Soda Ash Production</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.7  Soda Ash Production")</f>
+        <v>2.B.7  Soda Ash Production</v>
       </c>
       <c r="E59" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -5392,8 +5392,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D63" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.b. Ethylene")</f>
-        <v>2.B.8.b. Ethylene</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B.8.b  Ethylene")</f>
+        <v>2.B.8.b  Ethylene</v>
       </c>
       <c r="E63" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -5716,8 +5716,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D75" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.F Field Burning of Agricultural Residues")</f>
-        <v>3.F Field Burning of Agricultural Residues</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.F  Field Burning of Agricultural Residues")</f>
+        <v>3.F  Field Burning of Agricultural Residues</v>
       </c>
       <c r="E75" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -5743,8 +5743,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D76" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.D. Agricultural Soils")</f>
-        <v>3.D. Agricultural Soils</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.D  Agricultural Soils")</f>
+        <v>3.D  Agricultural Soils</v>
       </c>
       <c r="E76" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -5905,8 +5905,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D82" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.D. Agricultural Soils")</f>
-        <v>3.D. Agricultural Soils</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.D  Agricultural Soils")</f>
+        <v>3.D  Agricultural Soils</v>
       </c>
       <c r="E82" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -5932,8 +5932,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D83" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.F Field Burning of Agricultural Residues")</f>
-        <v>3.F Field Burning of Agricultural Residues</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.F  Field Burning of Agricultural Residues")</f>
+        <v>3.F  Field Burning of Agricultural Residues</v>
       </c>
       <c r="E83" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11009,8 +11009,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D3" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii Heat Plants")</f>
-        <v>1.A.1.a.iii Heat Plants</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii  Heat Plants")</f>
+        <v>1.A.1.a.iii  Heat Plants</v>
       </c>
       <c r="E3" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11045,8 +11045,8 @@
         <v>1</v>
       </c>
       <c r="B5" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aviation")</f>
-        <v>aviation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"domestic-aviation")</f>
+        <v>domestic-aviation</v>
       </c>
       <c r="C5" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
@@ -11067,8 +11067,8 @@
         <v>1</v>
       </c>
       <c r="B6" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"shipping")</f>
-        <v>shipping</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"domestic-shipping")</f>
+        <v>domestic-shipping</v>
       </c>
       <c r="C6" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
@@ -11185,8 +11185,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D11" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.v Distribution of Oil Products ")</f>
-        <v>1.B.2.a.v Distribution of Oil Products </v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.v  Distribution of Oil Products ")</f>
+        <v>1.B.2.a.v  Distribution of Oil Products </v>
       </c>
       <c r="E11" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11194,7 +11194,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9"/>
+      <c r="A12" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
+        <v>1</v>
+      </c>
       <c r="B12" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
@@ -11204,8 +11207,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D12" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi Other")</f>
-        <v>1.B.2.a.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi  Other")</f>
+        <v>1.B.2.a.vi  Other</v>
       </c>
       <c r="E12" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11213,7 +11216,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9"/>
+      <c r="A13" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
+        <v>1</v>
+      </c>
       <c r="B13" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
@@ -11223,8 +11229,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D13" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.v Distribution")</f>
-        <v>1.B.2.b.v Distribution</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.v  Distribution")</f>
+        <v>1.B.2.b.v  Distribution</v>
       </c>
       <c r="E13" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11232,7 +11238,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9"/>
+      <c r="A14" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
+        <v>1</v>
+      </c>
       <c r="B14" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
@@ -11242,8 +11251,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D14" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi Other")</f>
-        <v>1.B.2.b.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi  Other")</f>
+        <v>1.B.2.b.vi  Other</v>
       </c>
       <c r="E14" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11251,7 +11260,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9"/>
+      <c r="A15" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
+        <v>1</v>
+      </c>
       <c r="B15" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
@@ -11261,8 +11273,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D15" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.d Other")</f>
-        <v>1.B.2.d Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.d  Other")</f>
+        <v>1.B.2.d  Other</v>
       </c>
       <c r="E15" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11270,7 +11282,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9"/>
+      <c r="A16" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
+        <v>1</v>
+      </c>
       <c r="B16" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
@@ -11280,8 +11295,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D16" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c.ii Oil and Gas Extraction")</f>
-        <v>1.A.1.c.ii Oil and Gas Extraction</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c.ii  Oil and Gas Extraction")</f>
+        <v>1.A.1.c.ii  Oil and Gas Extraction</v>
       </c>
       <c r="E16" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11324,8 +11339,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D18" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c. Manufacture of Solid Fuels and Other Energy Industries")</f>
-        <v>1.A.1.c. Manufacture of Solid Fuels and Other Energy Industries</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c.  Manufacture of Solid Fuels and Other Energy Industries")</f>
+        <v>1.A.1.c.  Manufacture of Solid Fuels and Other Energy Industries</v>
       </c>
       <c r="E18" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11579,8 +11594,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D30" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b Non-Ferrous Metals")</f>
-        <v>1.A.2.b Non-Ferrous Metals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b  Non-Ferrous Metals")</f>
+        <v>1.A.2.b  Non-Ferrous Metals</v>
       </c>
       <c r="E30" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11601,8 +11616,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D31" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d Pulp, Paper and Print")</f>
-        <v>1.A.2.d Pulp, Paper and Print</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d  Pulp, Paper and Print")</f>
+        <v>1.A.2.d  Pulp, Paper and Print</v>
       </c>
       <c r="E31" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -11777,8 +11792,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D39" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d Pulp, Paper and Print")</f>
-        <v>1.A.2.d Pulp, Paper and Print</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d  Pulp, Paper and Print")</f>
+        <v>1.A.2.d  Pulp, Paper and Print</v>
       </c>
       <c r="E39" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -12770,38 +12785,65 @@
         <v>0</v>
       </c>
       <c r="B89" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"electricity-generation")</f>
+        <v>electricity-generation</v>
+      </c>
+      <c r="C89" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D89" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii  Heat Plants")</f>
+        <v>1.A.1.a.iii  Heat Plants</v>
+      </c>
+      <c r="E89" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B90" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"electricity-generation")</f>
+        <v>electricity-generation</v>
+      </c>
+      <c r="C90" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D90" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iv  Other")</f>
+        <v>1.A.1.a.iv  Other</v>
+      </c>
+      <c r="E90" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B91" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"domestic-aviation")</f>
         <v>domestic-aviation</v>
       </c>
-      <c r="C89" s="9"/>
-      <c r="D89" s="9"/>
-      <c r="E89" s="9"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B90" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"international-aviation")</f>
-        <v>international-aviation</v>
-      </c>
-      <c r="C90" s="9"/>
-      <c r="D90" s="9"/>
-      <c r="E90" s="9"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B91" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"international-shipping")</f>
-        <v>international-shipping</v>
-      </c>
-      <c r="C91" s="9"/>
-      <c r="D91" s="9"/>
-      <c r="E91" s="9"/>
+      <c r="C91" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D91" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.a Civil Aviation")</f>
+        <v>1.A.3.a Civil Aviation</v>
+      </c>
+      <c r="E91" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="b">
@@ -12812,9 +12854,18 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"domestic-shipping")</f>
         <v>domestic-shipping</v>
       </c>
-      <c r="C92" s="9"/>
-      <c r="D92" s="9"/>
-      <c r="E92" s="9"/>
+      <c r="C92" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D92" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.d Water-borne Navigation")</f>
+        <v>1.A.3.d Water-borne Navigation</v>
+      </c>
+      <c r="E92" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="9" t="b">
@@ -12825,9 +12876,18 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"coal-mining")</f>
         <v>coal-mining</v>
       </c>
-      <c r="C93" s="9"/>
-      <c r="D93" s="9"/>
-      <c r="E93" s="9"/>
+      <c r="C93" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D93" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.1 Solid Fuels")</f>
+        <v>1.B.1 Solid Fuels</v>
+      </c>
+      <c r="E93" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="b">
@@ -12835,160 +12895,214 @@
         <v>0</v>
       </c>
       <c r="B94" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"coal-mining")</f>
+        <v>coal-mining</v>
+      </c>
+      <c r="C94" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D94" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.1.b  Solid Fuel Transformation")</f>
+        <v>1.B.1.b  Solid Fuel Transformation</v>
+      </c>
+      <c r="E94" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B95" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"coal-mining")</f>
+        <v>coal-mining</v>
+      </c>
+      <c r="C95" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D95" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.1.c  Other")</f>
+        <v>1.B.1.c  Other</v>
+      </c>
+      <c r="E95" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B96" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
         <v>oil-and-gas-production-and-transport</v>
       </c>
-      <c r="C94" s="9" t="str">
+      <c r="C96" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
         <v>edgar</v>
       </c>
-      <c r="D94" s="9" t="str">
+      <c r="D96" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2 Oil and Natural Gas")</f>
         <v>1.B.2 Oil and Natural Gas</v>
       </c>
-      <c r="E94" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B95" s="9" t="str">
+      <c r="E96" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B97" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C97" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D97" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.v  Distribution of Oil Products ")</f>
+        <v>1.B.2.a.v  Distribution of Oil Products </v>
+      </c>
+      <c r="E97" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B98" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C98" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D98" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi  Other")</f>
+        <v>1.B.2.a.vi  Other</v>
+      </c>
+      <c r="E98" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B99" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C99" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D99" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.v  Distribution")</f>
+        <v>1.B.2.b.v  Distribution</v>
+      </c>
+      <c r="E99" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B100" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C100" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D100" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi  Other")</f>
+        <v>1.B.2.b.vi  Other</v>
+      </c>
+      <c r="E100" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B101" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C101" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D101" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.d  Other")</f>
+        <v>1.B.2.d  Other</v>
+      </c>
+      <c r="E101" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B102" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-production-and-transport")</f>
+        <v>oil-and-gas-production-and-transport</v>
+      </c>
+      <c r="C102" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D102" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c.ii  Oil and Gas Extraction")</f>
+        <v>1.A.1.c.ii  Oil and Gas Extraction</v>
+      </c>
+      <c r="E102" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B103" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-refining")</f>
         <v>oil-and-gas-refining</v>
-      </c>
-      <c r="C95" s="9"/>
-      <c r="D95" s="9"/>
-      <c r="E95" s="9"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B96" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"petrochemicals")</f>
-        <v>petrochemicals</v>
-      </c>
-      <c r="C96" s="9"/>
-      <c r="D96" s="9"/>
-      <c r="E96" s="9"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B97" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"cement")</f>
-        <v>cement</v>
-      </c>
-      <c r="C97" s="9"/>
-      <c r="D97" s="9"/>
-      <c r="E97" s="9"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B98" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"chemicals")</f>
-        <v>chemicals</v>
-      </c>
-      <c r="C98" s="9"/>
-      <c r="D98" s="9"/>
-      <c r="E98" s="9"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B99" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
-        <v>steel</v>
-      </c>
-      <c r="C99" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
-        <v>edgar</v>
-      </c>
-      <c r="D99" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C Metal Industry")</f>
-        <v>2.C Metal Industry</v>
-      </c>
-      <c r="E99" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B100" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
-        <v>aluminum</v>
-      </c>
-      <c r="C100" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
-        <v>edgar</v>
-      </c>
-      <c r="D100" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C Metal Industry")</f>
-        <v>2.C Metal Industry</v>
-      </c>
-      <c r="E100" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B101" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
-        <v>pulp-and-paper</v>
-      </c>
-      <c r="C101" s="9"/>
-      <c r="D101" s="9"/>
-      <c r="E101" s="9"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B102" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"mining-and-quarrying")</f>
-        <v>mining-and-quarrying</v>
-      </c>
-      <c r="C102" s="9"/>
-      <c r="D102" s="9"/>
-      <c r="E102" s="9"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B103" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
       </c>
       <c r="C103" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
         <v>edgar</v>
       </c>
       <c r="D103" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.bc Petroleum Refining - Manufacture of Solid Fuels and Other Energy Industries")</f>
+        <v>1.A.1.bc Petroleum Refining - Manufacture of Solid Fuels and Other Energy Industries</v>
       </c>
       <c r="E103" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -13001,16 +13115,16 @@
         <v>0</v>
       </c>
       <c r="B104" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"oil-and-gas-refining")</f>
+        <v>oil-and-gas-refining</v>
       </c>
       <c r="C104" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D104" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.c.  Manufacture of Solid Fuels and Other Energy Industries")</f>
+        <v>1.A.1.c.  Manufacture of Solid Fuels and Other Energy Industries</v>
       </c>
       <c r="E104" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13023,126 +13137,117 @@
         <v>0</v>
       </c>
       <c r="B105" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
-      </c>
-      <c r="C105" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
-      </c>
-      <c r="D105" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
-      </c>
-      <c r="E105" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"petrochemicals")</f>
+        <v>petrochemicals</v>
+      </c>
+      <c r="C105" s="9"/>
+      <c r="D105" s="9"/>
+      <c r="E105" s="9"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B106" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"cement")</f>
+        <v>cement</v>
+      </c>
+      <c r="C106" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D106" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.A.1 Cement production")</f>
+        <v>2.A.1 Cement production</v>
+      </c>
+      <c r="E106" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B107" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"chemicals")</f>
+        <v>chemicals</v>
+      </c>
+      <c r="C107" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D107" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.B Chemical Industry")</f>
+        <v>2.B Chemical Industry</v>
+      </c>
+      <c r="E107" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B108" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
+      </c>
+      <c r="C108" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D108" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C Metal Industry")</f>
+        <v>2.C Metal Industry</v>
+      </c>
+      <c r="E108" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B109" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
+      </c>
+      <c r="C109" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D109" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.3  Aluminium Production")</f>
+        <v>2.C.3  Aluminium Production</v>
+      </c>
+      <c r="E109" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
         <v>-1</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B106" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
-      </c>
-      <c r="C106" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
-      </c>
-      <c r="D106" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
-      </c>
-      <c r="E106" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B107" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
-      </c>
-      <c r="C107" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
-      </c>
-      <c r="D107" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
-      </c>
-      <c r="E107" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B108" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
-      </c>
-      <c r="C108" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
-      </c>
-      <c r="D108" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
-      </c>
-      <c r="E108" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B109" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
-      </c>
-      <c r="C109" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
-        <v>edgar</v>
-      </c>
-      <c r="D109" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
-      </c>
-      <c r="E109" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-    </row>
     <row r="110">
       <c r="A110" s="9" t="b">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
         <v>0</v>
       </c>
       <c r="B110" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C110" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D110" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.2  Ferroalloys Production")</f>
+        <v>2.C.2  Ferroalloys Production</v>
       </c>
       <c r="E110" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13155,16 +13260,16 @@
         <v>0</v>
       </c>
       <c r="B111" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C111" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D111" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.4  Magnesium Production")</f>
+        <v>2.C.4  Magnesium Production</v>
       </c>
       <c r="E111" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13177,16 +13282,16 @@
         <v>0</v>
       </c>
       <c r="B112" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C112" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D112" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.5  Lead Production")</f>
+        <v>2.C.5  Lead Production</v>
       </c>
       <c r="E112" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13199,16 +13304,16 @@
         <v>0</v>
       </c>
       <c r="B113" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C113" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D113" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.6  Zinc Production")</f>
+        <v>2.C.6  Zinc Production</v>
       </c>
       <c r="E113" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13221,16 +13326,16 @@
         <v>0</v>
       </c>
       <c r="B114" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C114" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D114" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.7  Other")</f>
+        <v>2.C.7  Other</v>
       </c>
       <c r="E114" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13243,16 +13348,16 @@
         <v>0</v>
       </c>
       <c r="B115" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C115" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
         <v>edgar</v>
       </c>
       <c r="D115" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2 Manufacturing Industries and Construction")</f>
+        <v>1.A.2 Manufacturing Industries and Construction</v>
       </c>
       <c r="E115" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -13265,16 +13370,16 @@
         <v>0</v>
       </c>
       <c r="B116" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C116" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D116" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b  Non-Ferrous Metals")</f>
+        <v>1.A.2.b  Non-Ferrous Metals</v>
       </c>
       <c r="E116" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13287,16 +13392,16 @@
         <v>0</v>
       </c>
       <c r="B117" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C117" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D117" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d  Pulp, Paper and Print")</f>
+        <v>1.A.2.d  Pulp, Paper and Print</v>
       </c>
       <c r="E117" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13309,16 +13414,16 @@
         <v>0</v>
       </c>
       <c r="B118" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C118" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D118" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
       </c>
       <c r="E118" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13331,16 +13436,16 @@
         <v>0</v>
       </c>
       <c r="B119" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C119" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D119" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.e  Food Processing, Beverages and Tobacco")</f>
+        <v>1.A.2.e  Food Processing, Beverages and Tobacco</v>
       </c>
       <c r="E119" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13353,16 +13458,16 @@
         <v>0</v>
       </c>
       <c r="B120" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C120" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D120" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.f  Non-metallic Minerals")</f>
+        <v>1.A.2.f  Non-metallic Minerals</v>
       </c>
       <c r="E120" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13375,42 +13480,42 @@
         <v>0</v>
       </c>
       <c r="B121" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"steel")</f>
+        <v>steel</v>
       </c>
       <c r="C121" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D121" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.g  Other")</f>
+        <v>1.A.2.g  Other</v>
+      </c>
+      <c r="E121" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B122" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
+      </c>
+      <c r="C122" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
         <v>edgar</v>
       </c>
-      <c r="D121" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
-      </c>
-      <c r="E121" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="B122" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
-      </c>
-      <c r="C122" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
-      </c>
       <c r="D122" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C Metal Industry")</f>
+        <v>2.C Metal Industry</v>
       </c>
       <c r="E122" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -13419,20 +13524,20 @@
         <v>0</v>
       </c>
       <c r="B123" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C123" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
       </c>
       <c r="D123" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2 Manufacturing Industries and Construction")</f>
+        <v>1.A.2 Manufacturing Industries and Construction</v>
       </c>
       <c r="E123" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -13441,16 +13546,16 @@
         <v>0</v>
       </c>
       <c r="B124" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C124" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D124" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.a  Iron and Steel")</f>
+        <v>1.A.2.a  Iron and Steel</v>
       </c>
       <c r="E124" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13463,16 +13568,16 @@
         <v>0</v>
       </c>
       <c r="B125" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C125" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D125" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d  Pulp, Paper and Print")</f>
+        <v>1.A.2.d  Pulp, Paper and Print</v>
       </c>
       <c r="E125" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13485,16 +13590,16 @@
         <v>0</v>
       </c>
       <c r="B126" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C126" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D126" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
       </c>
       <c r="E126" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13507,20 +13612,20 @@
         <v>0</v>
       </c>
       <c r="B127" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C127" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
-        <v>edgar</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D127" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.e  Food Processing, Beverages and Tobacco")</f>
+        <v>1.A.2.e  Food Processing, Beverages and Tobacco</v>
       </c>
       <c r="E127" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
       </c>
     </row>
     <row r="128">
@@ -13529,16 +13634,16 @@
         <v>0</v>
       </c>
       <c r="B128" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C128" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D128" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.f  Non-metallic Minerals")</f>
+        <v>1.A.2.f  Non-metallic Minerals</v>
       </c>
       <c r="E128" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13551,16 +13656,16 @@
         <v>0</v>
       </c>
       <c r="B129" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C129" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D129" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.g  Other")</f>
+        <v>1.A.2.g  Other</v>
       </c>
       <c r="E129" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13573,16 +13678,16 @@
         <v>0</v>
       </c>
       <c r="B130" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C130" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D130" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.1  Iron and Steel Production")</f>
+        <v>2.C.1  Iron and Steel Production</v>
       </c>
       <c r="E130" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13595,16 +13700,16 @@
         <v>0</v>
       </c>
       <c r="B131" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C131" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D131" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.2  Ferroalloys Production")</f>
+        <v>2.C.2  Ferroalloys Production</v>
       </c>
       <c r="E131" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13617,16 +13722,16 @@
         <v>0</v>
       </c>
       <c r="B132" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C132" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D132" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.4  Magnesium Production")</f>
+        <v>2.C.4  Magnesium Production</v>
       </c>
       <c r="E132" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13639,20 +13744,20 @@
         <v>0</v>
       </c>
       <c r="B133" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C133" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
-        <v>edgar</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D133" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
-        <v>3.A.1 Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.5  Lead Production")</f>
+        <v>2.C.5  Lead Production</v>
       </c>
       <c r="E133" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
       </c>
     </row>
     <row r="134">
@@ -13661,16 +13766,16 @@
         <v>0</v>
       </c>
       <c r="B134" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C134" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D134" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
-        <v>enteric-fermentation-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.6  Zinc Production")</f>
+        <v>2.C.6  Zinc Production</v>
       </c>
       <c r="E134" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13683,16 +13788,16 @@
         <v>0</v>
       </c>
       <c r="B135" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"aluminum")</f>
+        <v>aluminum</v>
       </c>
       <c r="C135" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D135" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
-        <v>manure-left-on-pasture-cattle</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.7  Other")</f>
+        <v>2.C.7  Other</v>
       </c>
       <c r="E135" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13705,20 +13810,20 @@
         <v>0</v>
       </c>
       <c r="B136" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
       </c>
       <c r="C136" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
       </c>
       <c r="D136" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
-        <v>manure-management-cattle-feedlot</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2 Manufacturing Industries and Construction")</f>
+        <v>1.A.2 Manufacturing Industries and Construction</v>
       </c>
       <c r="E136" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
-        <v>-1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -13727,16 +13832,16 @@
         <v>0</v>
       </c>
       <c r="B137" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
       </c>
       <c r="C137" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D137" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
-        <v>enteric-fermentation-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.a  Iron and Steel")</f>
+        <v>1.A.2.a  Iron and Steel</v>
       </c>
       <c r="E137" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13749,16 +13854,16 @@
         <v>0</v>
       </c>
       <c r="B138" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
-        <v>enteric-fermentation-cattle-pasture</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
       </c>
       <c r="C138" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
-        <v>climate-trace</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
       </c>
       <c r="D138" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
-        <v>manure-management-other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b  Non-Ferrous Metals")</f>
+        <v>1.A.2.b  Non-Ferrous Metals</v>
       </c>
       <c r="E138" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13771,12 +13876,21 @@
         <v>0</v>
       </c>
       <c r="B139" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"rice-cultivation")</f>
-        <v>rice-cultivation</v>
-      </c>
-      <c r="C139" s="9"/>
-      <c r="D139" s="9"/>
-      <c r="E139" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
+      </c>
+      <c r="C139" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D139" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
+      </c>
+      <c r="E139" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="9" t="b">
@@ -13784,12 +13898,21 @@
         <v>0</v>
       </c>
       <c r="B140" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"synthetic-fertilizer-application")</f>
-        <v>synthetic-fertilizer-application</v>
-      </c>
-      <c r="C140" s="9"/>
-      <c r="D140" s="9"/>
-      <c r="E140" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
+      </c>
+      <c r="C140" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D140" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.e  Food Processing, Beverages and Tobacco")</f>
+        <v>1.A.2.e  Food Processing, Beverages and Tobacco</v>
+      </c>
+      <c r="E140" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="9" t="b">
@@ -13797,12 +13920,21 @@
         <v>0</v>
       </c>
       <c r="B141" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-fires")</f>
-        <v>forest-land-fires</v>
-      </c>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9"/>
-      <c r="E141" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
+      </c>
+      <c r="C141" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D141" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.f  Non-metallic Minerals")</f>
+        <v>1.A.2.f  Non-metallic Minerals</v>
+      </c>
+      <c r="E141" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="9" t="b">
@@ -13810,12 +13942,21 @@
         <v>0</v>
       </c>
       <c r="B142" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-clearing")</f>
-        <v>forest-land-clearing</v>
-      </c>
-      <c r="C142" s="9"/>
-      <c r="D142" s="9"/>
-      <c r="E142" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"pulp-and-paper")</f>
+        <v>pulp-and-paper</v>
+      </c>
+      <c r="C142" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"unfccc_non_annex_1")</f>
+        <v>unfccc_non_annex_1</v>
+      </c>
+      <c r="D142" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.g  Other")</f>
+        <v>1.A.2.g  Other</v>
+      </c>
+      <c r="E142" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="9" t="b">
@@ -13823,8 +13964,8 @@
         <v>0</v>
       </c>
       <c r="B143" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-degradation")</f>
-        <v>forest-land-degradation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"mining-and-quarrying")</f>
+        <v>mining-and-quarrying</v>
       </c>
       <c r="C143" s="9"/>
       <c r="D143" s="9"/>
@@ -13836,12 +13977,21 @@
         <v>0</v>
       </c>
       <c r="B144" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-forest-land")</f>
-        <v>net-forest-land</v>
-      </c>
-      <c r="C144" s="9"/>
-      <c r="D144" s="9"/>
-      <c r="E144" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
+        <v>enteric-fermentation-cattle-feedlot</v>
+      </c>
+      <c r="C144" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D144" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
+        <v>3.A.1 Enteric Fermentation</v>
+      </c>
+      <c r="E144" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="9" t="b">
@@ -13849,12 +13999,21 @@
         <v>0</v>
       </c>
       <c r="B145" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-shrubgrass")</f>
-        <v>net-shrubgrass</v>
-      </c>
-      <c r="C145" s="9"/>
-      <c r="D145" s="9"/>
-      <c r="E145" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
+        <v>enteric-fermentation-cattle-feedlot</v>
+      </c>
+      <c r="C145" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D145" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
+        <v>enteric-fermentation-cattle-pasture</v>
+      </c>
+      <c r="E145" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="9" t="b">
@@ -13862,12 +14021,21 @@
         <v>0</v>
       </c>
       <c r="B146" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-wetland")</f>
-        <v>net-wetland</v>
-      </c>
-      <c r="C146" s="9"/>
-      <c r="D146" s="9"/>
-      <c r="E146" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
+        <v>enteric-fermentation-cattle-feedlot</v>
+      </c>
+      <c r="C146" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D146" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
+        <v>enteric-fermentation-other</v>
+      </c>
+      <c r="E146" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="9" t="b">
@@ -13875,12 +14043,21 @@
         <v>0</v>
       </c>
       <c r="B147" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"shrubgrass-fires")</f>
-        <v>shrubgrass-fires</v>
-      </c>
-      <c r="C147" s="9"/>
-      <c r="D147" s="9"/>
-      <c r="E147" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
+        <v>manure-left-on-pasture-cattle</v>
+      </c>
+      <c r="C147" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D147" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.2 Manure Management")</f>
+        <v>3.A.2 Manure Management</v>
+      </c>
+      <c r="E147" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="9" t="b">
@@ -13888,12 +14065,21 @@
         <v>0</v>
       </c>
       <c r="B148" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"wetland-fires")</f>
-        <v>wetland-fires</v>
-      </c>
-      <c r="C148" s="9"/>
-      <c r="D148" s="9"/>
-      <c r="E148" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
+        <v>manure-left-on-pasture-cattle</v>
+      </c>
+      <c r="C148" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D148" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
+        <v>manure-management-cattle-feedlot</v>
+      </c>
+      <c r="E148" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="9" t="b">
@@ -13901,12 +14087,21 @@
         <v>0</v>
       </c>
       <c r="B149" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"removals")</f>
-        <v>removals</v>
-      </c>
-      <c r="C149" s="9"/>
-      <c r="D149" s="9"/>
-      <c r="E149" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
+        <v>manure-left-on-pasture-cattle</v>
+      </c>
+      <c r="C149" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D149" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
+        <v>manure-management-other</v>
+      </c>
+      <c r="E149" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="9" t="b">
@@ -13914,170 +14109,434 @@
         <v>0</v>
       </c>
       <c r="B150" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"water-reservoirs")</f>
-        <v>water-reservoirs</v>
-      </c>
-      <c r="C150" s="9"/>
-      <c r="D150" s="9"/>
-      <c r="E150" s="9"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
+        <v>manure-management-cattle-feedlot</v>
+      </c>
+      <c r="C150" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D150" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.2 Manure Management")</f>
+        <v>3.A.2 Manure Management</v>
+      </c>
+      <c r="E150" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="9"/>
-      <c r="B151" s="9"/>
-      <c r="C151" s="9"/>
-      <c r="D151" s="9"/>
-      <c r="E151" s="9"/>
+      <c r="A151" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B151" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
+        <v>manure-management-cattle-feedlot</v>
+      </c>
+      <c r="C151" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D151" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
+        <v>manure-left-on-pasture-cattle</v>
+      </c>
+      <c r="E151" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" s="9"/>
-      <c r="B152" s="9"/>
-      <c r="C152" s="9"/>
-      <c r="D152" s="9"/>
-      <c r="E152" s="9"/>
+      <c r="A152" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B152" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
+        <v>manure-management-cattle-feedlot</v>
+      </c>
+      <c r="C152" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D152" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
+        <v>manure-management-other</v>
+      </c>
+      <c r="E152" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="9"/>
-      <c r="B153" s="9"/>
-      <c r="C153" s="9"/>
-      <c r="D153" s="9"/>
-      <c r="E153" s="9"/>
+      <c r="A153" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B153" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
+        <v>enteric-fermentation-other</v>
+      </c>
+      <c r="C153" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D153" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
+        <v>3.A.1 Enteric Fermentation</v>
+      </c>
+      <c r="E153" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" s="9"/>
-      <c r="B154" s="9"/>
-      <c r="C154" s="9"/>
-      <c r="D154" s="9"/>
-      <c r="E154" s="9"/>
+      <c r="A154" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B154" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
+        <v>enteric-fermentation-other</v>
+      </c>
+      <c r="C154" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D154" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
+        <v>enteric-fermentation-cattle-feedlot</v>
+      </c>
+      <c r="E154" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="9"/>
-      <c r="B155" s="9"/>
-      <c r="C155" s="9"/>
-      <c r="D155" s="9"/>
-      <c r="E155" s="9"/>
+      <c r="A155" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B155" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
+        <v>enteric-fermentation-other</v>
+      </c>
+      <c r="C155" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D155" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
+        <v>enteric-fermentation-cattle-pasture</v>
+      </c>
+      <c r="E155" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" s="9"/>
-      <c r="B156" s="9"/>
-      <c r="C156" s="9"/>
-      <c r="D156" s="9"/>
-      <c r="E156" s="9"/>
+      <c r="A156" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B156" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
+        <v>manure-management-other</v>
+      </c>
+      <c r="C156" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D156" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.2 Manure Management")</f>
+        <v>3.A.2 Manure Management</v>
+      </c>
+      <c r="E156" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="9"/>
-      <c r="B157" s="9"/>
-      <c r="C157" s="9"/>
-      <c r="D157" s="9"/>
-      <c r="E157" s="9"/>
+      <c r="A157" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B157" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
+        <v>manure-management-other</v>
+      </c>
+      <c r="C157" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D157" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
+        <v>manure-left-on-pasture-cattle</v>
+      </c>
+      <c r="E157" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" s="9"/>
-      <c r="B158" s="9"/>
-      <c r="C158" s="9"/>
-      <c r="D158" s="9"/>
-      <c r="E158" s="9"/>
+      <c r="A158" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B158" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
+        <v>manure-management-other</v>
+      </c>
+      <c r="C158" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D158" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
+        <v>manure-management-cattle-feedlot</v>
+      </c>
+      <c r="E158" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="9"/>
-      <c r="B159" s="9"/>
-      <c r="C159" s="9"/>
-      <c r="D159" s="9"/>
-      <c r="E159" s="9"/>
+      <c r="A159" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B159" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
+        <v>enteric-fermentation-cattle-pasture</v>
+      </c>
+      <c r="C159" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D159" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A.1 Enteric Fermentation")</f>
+        <v>3.A.1 Enteric Fermentation</v>
+      </c>
+      <c r="E159" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="9"/>
-      <c r="B160" s="9"/>
-      <c r="C160" s="9"/>
-      <c r="D160" s="9"/>
-      <c r="E160" s="9"/>
+      <c r="A160" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B160" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
+        <v>enteric-fermentation-cattle-pasture</v>
+      </c>
+      <c r="C160" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D160" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
+        <v>enteric-fermentation-cattle-feedlot</v>
+      </c>
+      <c r="E160" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" s="9"/>
-      <c r="B161" s="9"/>
-      <c r="C161" s="9"/>
-      <c r="D161" s="9"/>
-      <c r="E161" s="9"/>
+      <c r="A161" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B161" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
+        <v>enteric-fermentation-cattle-pasture</v>
+      </c>
+      <c r="C161" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"climate-trace")</f>
+        <v>climate-trace</v>
+      </c>
+      <c r="D161" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
+        <v>enteric-fermentation-other</v>
+      </c>
+      <c r="E161" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
+        <v>-1</v>
+      </c>
     </row>
     <row r="162">
-      <c r="A162" s="9"/>
-      <c r="B162" s="9"/>
-      <c r="C162" s="9"/>
-      <c r="D162" s="9"/>
-      <c r="E162" s="9"/>
+      <c r="A162" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B162" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"rice-cultivation")</f>
+        <v>rice-cultivation</v>
+      </c>
+      <c r="C162" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D162" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C.7 Rice cultivations")</f>
+        <v>3.C.7 Rice cultivations</v>
+      </c>
+      <c r="E162" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="163">
-      <c r="A163" s="9"/>
-      <c r="B163" s="9"/>
-      <c r="C163" s="9"/>
-      <c r="D163" s="9"/>
-      <c r="E163" s="9"/>
+      <c r="A163" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B163" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"synthetic-fertilizer-application")</f>
+        <v>synthetic-fertilizer-application</v>
+      </c>
+      <c r="C163" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"edgar")</f>
+        <v>edgar</v>
+      </c>
+      <c r="D163" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C.4 Direct N2O Emissions from managed soils")</f>
+        <v>3.C.4 Direct N2O Emissions from managed soils</v>
+      </c>
+      <c r="E163" s="9">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" s="9"/>
-      <c r="B164" s="9"/>
+      <c r="A164" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B164" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-fires")</f>
+        <v>forest-land-fires</v>
+      </c>
       <c r="C164" s="9"/>
       <c r="D164" s="9"/>
       <c r="E164" s="9"/>
     </row>
     <row r="165">
-      <c r="A165" s="9"/>
-      <c r="B165" s="9"/>
+      <c r="A165" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B165" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-clearing")</f>
+        <v>forest-land-clearing</v>
+      </c>
       <c r="C165" s="9"/>
       <c r="D165" s="9"/>
       <c r="E165" s="9"/>
     </row>
     <row r="166">
-      <c r="A166" s="9"/>
-      <c r="B166" s="9"/>
+      <c r="A166" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B166" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"forest-land-degradation")</f>
+        <v>forest-land-degradation</v>
+      </c>
       <c r="C166" s="9"/>
       <c r="D166" s="9"/>
       <c r="E166" s="9"/>
     </row>
     <row r="167">
-      <c r="A167" s="9"/>
-      <c r="B167" s="9"/>
+      <c r="A167" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B167" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-forest-land")</f>
+        <v>net-forest-land</v>
+      </c>
       <c r="C167" s="9"/>
       <c r="D167" s="9"/>
       <c r="E167" s="9"/>
     </row>
     <row r="168">
-      <c r="A168" s="9"/>
-      <c r="B168" s="9"/>
+      <c r="A168" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B168" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-shrubgrass")</f>
+        <v>net-shrubgrass</v>
+      </c>
       <c r="C168" s="9"/>
       <c r="D168" s="9"/>
       <c r="E168" s="9"/>
     </row>
     <row r="169">
-      <c r="A169" s="9"/>
-      <c r="B169" s="9"/>
+      <c r="A169" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B169" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"net-wetland")</f>
+        <v>net-wetland</v>
+      </c>
       <c r="C169" s="9"/>
       <c r="D169" s="9"/>
       <c r="E169" s="9"/>
     </row>
     <row r="170">
-      <c r="A170" s="9"/>
-      <c r="B170" s="9"/>
+      <c r="A170" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B170" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"shrubgrass-fires")</f>
+        <v>shrubgrass-fires</v>
+      </c>
       <c r="C170" s="9"/>
       <c r="D170" s="9"/>
       <c r="E170" s="9"/>
     </row>
     <row r="171">
-      <c r="A171" s="9"/>
-      <c r="B171" s="9"/>
+      <c r="A171" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B171" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"wetland-fires")</f>
+        <v>wetland-fires</v>
+      </c>
       <c r="C171" s="9"/>
       <c r="D171" s="9"/>
       <c r="E171" s="9"/>
     </row>
     <row r="172">
-      <c r="A172" s="9"/>
-      <c r="B172" s="9"/>
+      <c r="A172" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B172" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"removals")</f>
+        <v>removals</v>
+      </c>
       <c r="C172" s="9"/>
       <c r="D172" s="9"/>
       <c r="E172" s="9"/>
     </row>
     <row r="173">
-      <c r="A173" s="9"/>
-      <c r="B173" s="9"/>
+      <c r="A173" s="9" t="b">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="B173" s="9" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"water-reservoirs")</f>
+        <v>water-reservoirs</v>
+      </c>
       <c r="C173" s="9"/>
       <c r="D173" s="9"/>
       <c r="E173" s="9"/>

</xml_diff>

<commit_message>
fixing aluminum in comp dictionary
</commit_message>
<xml_diff>
--- a/climate_trace_tools/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
+++ b/climate_trace_tools/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
@@ -4933,8 +4933,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D46" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.3  Aluminum Production")</f>
-        <v>2.C.3  Aluminum Production</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"2.C.3  Aluminium Production")</f>
+        <v>2.C.3  Aluminium Production</v>
       </c>
       <c r="E46" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>

</xml_diff>